<commit_message>
Fix contact-demo template for request-demo and other contact pages
Add cards-testimonial, logo-wall, and form parsers to the contact-demo import
script. Add sections transformer with 6 section definitions for proper section
breaks and backgrounds. Re-import all 3 contact-demo pages. The request-demo
page now renders testimonial cards, logo wall, and CTA banner with gradient.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-contact-demo.report.xlsx
+++ b/tools/importer/reports/import-contact-demo.report.xlsx
@@ -73,7 +73,7 @@
     <t>training-certification</t>
   </si>
   <si>
-    <t>2026-03-28T19:39:53.753Z</t>
+    <t>2026-03-28T22:28:18.683Z</t>
   </si>
   <si>
     <t>Cvent Academy | Cvent</t>
@@ -130,7 +130,7 @@
     <t>resource-listing</t>
   </si>
   <si>
-    <t>2026-03-28T19:38:05.603Z</t>
+    <t>2026-03-28T22:27:45.370Z</t>
   </si>
   <si>
     <t>Your Hub for Meetings, Hospitality, and Event Excellence | Cvent Blog</t>
@@ -148,7 +148,7 @@
     <t>en/case-studies</t>
   </si>
   <si>
-    <t>2026-03-28T19:38:11.569Z</t>
+    <t>2026-03-28T22:27:51.514Z</t>
   </si>
   <si>
     <t>Cvent Customer Success Stories &amp; Reviews</t>
@@ -184,7 +184,7 @@
     <t>contact-demo</t>
   </si>
   <si>
-    <t>2026-03-28T22:27:02.879Z</t>
+    <t>2026-03-29T22:58:58.559Z</t>
   </si>
   <si>
     <t>Contact Us | Cvent</t>
@@ -199,7 +199,7 @@
     <t>en/cvent-certification</t>
   </si>
   <si>
-    <t>2026-03-28T19:40:02.106Z</t>
+    <t>2026-03-28T22:28:27.045Z</t>
   </si>
   <si>
     <t>Cvent Certification | Cvent</t>
@@ -217,7 +217,7 @@
     <t>en/cvent-news-and-press-releases</t>
   </si>
   <si>
-    <t>2026-03-28T19:38:31.447Z</t>
+    <t>2026-03-28T22:28:13.765Z</t>
   </si>
   <si>
     <t>Cvent News &amp; Press Releases | Newsroom | Cvent</t>
@@ -229,7 +229,7 @@
     <t>en/cventiq.report.json</t>
   </si>
   <si>
-    <t>["columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial"]</t>
+    <t>["columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial","cards-testimonial","cards-feature"]</t>
   </si>
   <si>
     <t>en/cventiq</t>
@@ -238,7 +238,7 @@
     <t>product-platform</t>
   </si>
   <si>
-    <t>2026-03-28T22:25:34.453Z</t>
+    <t>2026-03-29T22:23:24.548Z</t>
   </si>
   <si>
     <t>CventIQ: AI Solutions for Events</t>
@@ -250,13 +250,13 @@
     <t>en/event-management-software.report.json</t>
   </si>
   <si>
-    <t>["hero-product-form","tabs-integrations","columns-media","cards-testimonial"]</t>
+    <t>["hero-product-form","tabs-integrations","columns-media","cards-testimonial","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall"]</t>
   </si>
   <si>
     <t>en/event-management-software</t>
   </si>
   <si>
-    <t>2026-03-28T22:24:54.167Z</t>
+    <t>2026-03-29T22:22:47.616Z</t>
   </si>
   <si>
     <t>Online Event Management Software | Cvent</t>
@@ -268,24 +268,24 @@
     <t>en/event-types.report.json</t>
   </si>
   <si>
+    <t>en/event-types</t>
+  </si>
+  <si>
+    <t>2026-03-29T22:23:17.222Z</t>
+  </si>
+  <si>
+    <t>404 | Cvent</t>
+  </si>
+  <si>
+    <t>https://www.cvent.com/en/event-types</t>
+  </si>
+  <si>
+    <t>en/management-team.report.json</t>
+  </si>
+  <si>
     <t>[]</t>
   </si>
   <si>
-    <t>en/event-types</t>
-  </si>
-  <si>
-    <t>2026-03-28T22:25:26.079Z</t>
-  </si>
-  <si>
-    <t>404 | Cvent</t>
-  </si>
-  <si>
-    <t>https://www.cvent.com/en/event-types</t>
-  </si>
-  <si>
-    <t>en/management-team.report.json</t>
-  </si>
-  <si>
     <t>en/management-team</t>
   </si>
   <si>
@@ -307,7 +307,7 @@
     <t>legal</t>
   </si>
   <si>
-    <t>2026-03-28T19:39:27.745Z</t>
+    <t>2026-03-28T22:27:16.161Z</t>
   </si>
   <si>
     <t>Cvent Privacy Policy | Cvent</t>
@@ -322,7 +322,7 @@
     <t>en/product-terms-of-use</t>
   </si>
   <si>
-    <t>2026-03-28T19:39:34.504Z</t>
+    <t>2026-03-28T22:27:21.983Z</t>
   </si>
   <si>
     <t>Terms of Use for Cvent Products | Cvent</t>
@@ -340,7 +340,7 @@
     <t>en/products</t>
   </si>
   <si>
-    <t>2026-03-28T22:25:19.343Z</t>
+    <t>2026-03-29T22:23:10.106Z</t>
   </si>
   <si>
     <t>Events &amp; Venue Management Products | Cvent</t>
@@ -352,13 +352,13 @@
     <t>en/request-demo.report.json</t>
   </si>
   <si>
-    <t>["hero-product-form"]</t>
+    <t>["hero-product-form","cards-testimonial","logo-wall"]</t>
   </si>
   <si>
     <t>en/request-demo</t>
   </si>
   <si>
-    <t>2026-03-28T22:26:54.796Z</t>
+    <t>2026-03-29T22:58:53.181Z</t>
   </si>
   <si>
     <t>Cvent Demo | Cvent</t>
@@ -373,7 +373,7 @@
     <t>en/resources</t>
   </si>
   <si>
-    <t>2026-03-28T19:38:26.017Z</t>
+    <t>2026-03-28T22:28:06.524Z</t>
   </si>
   <si>
     <t>Content Library | Resources | Cvent</t>
@@ -427,7 +427,7 @@
     <t>en/upcoming-webinars</t>
   </si>
   <si>
-    <t>2026-03-28T19:38:17.968Z</t>
+    <t>2026-03-28T22:28:00.140Z</t>
   </si>
   <si>
     <t>Upcoming Events</t>
@@ -442,7 +442,7 @@
     <t>en/website-terms-use</t>
   </si>
   <si>
-    <t>2026-03-28T19:39:41.775Z</t>
+    <t>2026-03-28T22:27:27.800Z</t>
   </si>
   <si>
     <t>Website Terms of Use | Cvent</t>
@@ -457,7 +457,7 @@
     <t>en/company/legal</t>
   </si>
   <si>
-    <t>2026-03-28T19:39:47.502Z</t>
+    <t>2026-03-28T22:27:33.832Z</t>
   </si>
   <si>
     <t>Cvent Legal</t>
@@ -472,7 +472,7 @@
     <t>en/contact/support</t>
   </si>
   <si>
-    <t>2026-03-28T22:27:10.203Z</t>
+    <t>2026-03-29T22:59:05.601Z</t>
   </si>
   <si>
     <t>Cvent Support</t>
@@ -484,13 +484,13 @@
     <t>en/event-management-software/cvent-integrations.report.json</t>
   </si>
   <si>
-    <t>["hero-product-form","tabs-integrations","columns-media","columns-media","columns-media","columns-media"]</t>
+    <t>["hero-product-form","tabs-integrations","columns-media","columns-media","columns-media","columns-media","columns-media","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall","logo-wall"]</t>
   </si>
   <si>
     <t>en/event-management-software/cvent-integrations</t>
   </si>
   <si>
-    <t>2026-03-28T22:25:01.555Z</t>
+    <t>2026-03-29T22:22:54.126Z</t>
   </si>
   <si>
     <t>Meeting &amp; Events Tools Integration With Cvent</t>
@@ -502,13 +502,13 @@
     <t>en/event-management-software/cvent-pricing.report.json</t>
   </si>
   <si>
-    <t>["cards-testimonial","cards-testimonial","cards-testimonial"]</t>
+    <t>["columns-media","columns-media","cards-testimonial","cards-testimonial","cards-testimonial","cards-feature","form","logo-wall"]</t>
   </si>
   <si>
     <t>en/event-management-software/cvent-pricing</t>
   </si>
   <si>
-    <t>2026-03-28T22:25:08.947Z</t>
+    <t>2026-03-29T22:23:03.109Z</t>
   </si>
   <si>
     <t>Cvent Pricing | Request a Quote</t>
@@ -742,7 +742,7 @@
     <t>resource-detail</t>
   </si>
   <si>
-    <t>2026-03-28T19:40:08.779Z</t>
+    <t>2026-03-28T22:27:40.483Z</t>
   </si>
   <si>
     <t>Your Top Event Trends for 2026 | Cvent</t>
@@ -1489,10 +1489,10 @@
         <v>84</v>
       </c>
       <c r="B14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" t="s">
         <v>85</v>
-      </c>
-      <c r="C14" t="s">
-        <v>86</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
@@ -1501,21 +1501,21 @@
         <v>74</v>
       </c>
       <c r="F14" t="s">
+        <v>86</v>
+      </c>
+      <c r="G14" t="s">
         <v>87</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>88</v>
-      </c>
-      <c r="H14" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>89</v>
+      </c>
+      <c r="B15" t="s">
         <v>90</v>
-      </c>
-      <c r="B15" t="s">
-        <v>85</v>
       </c>
       <c r="C15" t="s">
         <v>91</v>
@@ -1723,7 +1723,7 @@
         <v>136</v>
       </c>
       <c r="B23" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C23" t="s">
         <v>137</v>
@@ -1749,7 +1749,7 @@
         <v>141</v>
       </c>
       <c r="B24" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C24" t="s">
         <v>142</v>
@@ -2191,7 +2191,7 @@
         <v>240</v>
       </c>
       <c r="B41" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C41" t="s">
         <v>241</v>

</xml_diff>

<commit_message>
Add interactive form to hero-product-form block
Modify hero-product-form parser to generate fallback form field definitions
when Marketo form fields are not in the DOM (loaded via JS). Update block JS
to parse pipe-delimited field definitions and build interactive form with
labels, inputs, selects, and submit button. Add CSS for form styling within
the hero sidebar. Re-import request-demo and event-management-software pages.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-contact-demo.report.xlsx
+++ b/tools/importer/reports/import-contact-demo.report.xlsx
@@ -184,7 +184,7 @@
     <t>contact-demo</t>
   </si>
   <si>
-    <t>2026-03-29T22:58:58.559Z</t>
+    <t>2026-03-29T23:21:04.834Z</t>
   </si>
   <si>
     <t>Contact Us | Cvent</t>
@@ -358,7 +358,7 @@
     <t>en/request-demo</t>
   </si>
   <si>
-    <t>2026-03-29T22:58:53.181Z</t>
+    <t>2026-03-29T23:20:57.801Z</t>
   </si>
   <si>
     <t>Cvent Demo | Cvent</t>
@@ -472,7 +472,7 @@
     <t>en/contact/support</t>
   </si>
   <si>
-    <t>2026-03-29T22:59:05.601Z</t>
+    <t>2026-03-29T23:21:10.656Z</t>
   </si>
   <si>
     <t>Cvent Support</t>

</xml_diff>